<commit_message>
Fix empty watershed folders not tracked in git
Git ignores empty directories, so 76 watersheds with no downloaded PDFs
had no folder in the repository after clone. Each watershed folder now
includes a .gitkeep placeholder (243 folders, one per Literature.xlsx row).

- ensure_watershed_folder writes .gitkeep on create
- build_watershed_folder_map assigns unique folder per watershed row
- PDF_Library_Folder column added to Literature.xlsx
- scripts/ensure_watershed_folders.py for one-shot folder sync

Co-authored-by: SherryYoYo6 <SherryYoYo6@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Literature.xlsx
+++ b/Literature.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P244"/>
+  <dimension ref="A1:Q244"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -497,6 +497,11 @@
           <t>Missing_PDF_Citations</t>
         </is>
       </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>PDF_Library_Folder</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -559,6 +564,11 @@
           <t>Allen, P.M., Harmel, R.D., Arnold, J., Plant, B., Yelderman, J., King, K., 2005. Field data and flow system response in clay (vertisol) shale terrain, north central Texas, USA. Hydrol. Process. Int. J. 19, 2719â€“2736.</t>
         </is>
       </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Blacklands</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -619,6 +629,11 @@
         </is>
       </c>
       <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>CB1</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -689,6 +704,11 @@
 Giertz, S., DiekkrÃ¼ger, B. and Steup, G., 2006. Physically-based modelling of hydrological processes in a tropical headwater catchment (West Africa)â€“process representation and multi-criteria validation. Hydrology and Earth System Sciences, 10(6), pp.829-847.</t>
         </is>
       </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Aguima</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -785,6 +805,11 @@
 Tang, Q., Duncan, J.M., Guo, L., Lin, H., Xiao, D., Eissenstat, D.M., 2020. On the controls of preferential flow in soils of different hillslope position and lithological origin. Hydrological Processes 34, 42954306. https://doi.org/10.1002/hyp.13883</t>
         </is>
       </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Shale_Hills</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -847,6 +872,11 @@
           <t>Cain, Molly R, Dong Kook Woo, Praveen Kumar, Laura Keefer, and Adam S Ward, 2022. â€œAntecedent Conditions Control Thresholds of Tile-Runoff Generation and Nitrogen Export in Intensively Managed Landscapes.â€ Water Resources Research 58, no. 2 (2022): e2021WR030507.</t>
         </is>
       </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>IML_CZO</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -911,6 +941,11 @@
           <t>Calderon H, Uhlenbrook S. 2016. Characterizing the climatic water balance dynamics and different runoff components in a poorly gauged tropical forested catchment, Nicaragua. Hydrological Sciences Journal 61 (14): 2465â€“2480 DOI: 10.1080/02626667.2014.964244</t>
         </is>
       </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Rompeviento_and_El_Nancite</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -975,6 +1010,11 @@
           <t>Casper MC, Volkmann HN, Waldenmeyer G, Plate EJ. 2003. The separation of flow pathways in a sandstone catchment of the Northern Black Forest using DOC and a nested Approach. Physics and Chemistry of the Earth, Parts A/B/C 28 (6): 269â€“275 DOI: 10.1016/S1474-7065(03)00037-8</t>
         </is>
       </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Duerreychbachtal</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1037,6 +1077,11 @@
           <t>Dwivedi R, Meixner T, McIntosh JC, FerrÃ© PAT, Eastoe CJ, Niu G-Y, Minor RL, Barronâ€Gafford GA, Chorover J. 2019. Hydrologic functioning of the deep critical zone and contributions to streamflow in a highâ€elevation catchment: Testing of multiple conceptual models. Hydrological processes 33 (4): 476â€“494 DOI: 10.1002/hyp.13363</t>
         </is>
       </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Marshall_Gulch</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1103,6 +1148,11 @@
           <t>Exner-Kittridge M, Strauss P, BlÃ¶schl G, Eder A, Saracevic E, Zessner M. 2016. The seasonal dynamics of the stream sources and input flow paths of water and nitrogen of an Austrian headwater agricultural catchment. The Science of the total environment 542 (Pt A): 935â€“945 DOI: 10.1016/j.scitotenv.2015.10.151</t>
         </is>
       </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>HOAL_Petzenkirchen</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1165,6 +1215,11 @@
           <t>Flint AL, Flint LE, Bodvarsson GS, Kwicklis EM, Fabryka-Martin J. 2001. Evolution of the conceptual model of unsaturated zone hydrology at Yucca Mountain, Nevada. Journal of Hydrology 247 (1)</t>
         </is>
       </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Yucca_Mountain</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1223,6 +1278,11 @@
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Kerrien</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1311,6 +1371,11 @@
 McGlynn, B.L., McDonnel, J.J., Brammer, D.D., 2002. A review of the evolving perceptual model of hillslope flowpaths at the Maimai catchments, New Zealand. Journal of Hydrology 257 1-4.https://doi.org/10.1016/S0022-1694(01)00559-5</t>
         </is>
       </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Maimai_M8</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1403,6 +1468,11 @@
 Hudson, D.T., Leach, J.A., Webster, K., Houle, D., 2021. Streamflow regime of a lake?stream system based on long?term data from a high?density hydrometric network. Hydrological Processes 35, e14396. https://doi.org/10.1002/hyp.14396</t>
         </is>
       </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>WS10</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1467,6 +1537,11 @@
           <t>Gibson JJ, Yi Y, Birks SJ. 2016. Isotope-based partitioning of streamflow in the oil sands region, northern Alberta: Towards a monitoring strategy for assessing flow sources and water quality controls. Journal of Hydrology: Regional Studies 5: 131â€“148 DOI: 10.1016/j.ejrh.2015.12.062</t>
         </is>
       </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Athabasca_Oil_Sands_region</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1525,6 +1600,11 @@
         </is>
       </c>
       <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Pedler_Creek</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1589,6 +1669,11 @@
           <t>Hangen E, Lindenlaub M, Leibundgut C, von Wilpert K. 2001. Investigating mechanisms of stormflow generation by natural tracers and hydrometric data: a small catchment study in the Black Forest, Germany. Hydrological processes 15 (2): 183â€“199 DOI: 10.1002/hyp.142</t>
         </is>
       </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Conventwald</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1651,6 +1736,11 @@
           <t>Hartmann, A., Wagener, T., Rimmer, A., Lange, J., Brielmann, H., Weiler, M., 2013. Testing the realism of model structures to identify karst system processes using water quality and quantity signatures. Water Resour. Res. 49, 3345â€“3358.</t>
         </is>
       </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Mt_Hermon_Range</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1715,6 +1805,11 @@
           <t>Heller K, Kleber A. 2016. Hillslope runoff generation influenced by layered subsurface in a headwater catchment in Ore Mountains, Germany. Environmental Earth Sciences 75 (11): 943 DOI: 10.1007/s12665-016-5750-y</t>
         </is>
       </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>Freiberger_Mulde</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1773,6 +1868,11 @@
         </is>
       </c>
       <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>Kostroma</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1837,6 +1937,11 @@
           <t>Inamdar SP, Mitchell MJ. 2007. Contributions of riparian and hillslope waters to storm runoff across multiple catchments and storm events in a glaciated forested watershed. Journal of Hydrology 341 (1): 116â€“130 DOI: 10.1016/j.jhydrol.2007.05.007</t>
         </is>
       </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>Point_Peter_Brook</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1909,6 +2014,11 @@
           <t>Du, E., Link, T.E., Gravelle, J.A., Hubbart, J.A., 2014. Validation and sensitivity test of the distributed hydrology soil-vegetation model (DHSVM) in a forested mountain watershed. Hydrological Processes 28, 61966210. https://doi.org/10.1002/hyp.10110</t>
         </is>
       </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>3_watersheds_R</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1989,6 +2099,11 @@
           <t>Wenninger, Jochen, Stefan Uhlenbrook, Nils Tilch, and Christian Leibundgut, 2004. â€œExperimental Evidence of Fast Groundwater Responses in a Hillslope/Floodplain Area in the Black Forest Mountains, Germany.â€ Hydrological Processes 18, no. 17 (2004): 3305â€“22.</t>
         </is>
       </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>Brugga</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2067,6 +2182,11 @@
 Tang, Q., Duncan, J.M., Guo, L., Lin, H., Xiao, D., Eissenstat, D.M., 2020. On the controls of preferential flow in soils of different hillslope position and lithological origin. Hydrological Processes 34, 42954306. https://doi.org/10.1002/hyp.13883</t>
         </is>
       </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>Garner_Run</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2145,6 +2265,11 @@
 Lin, H.S., Kogelmann, W., Walker, C., Bruns, M.A., 2006. Soil moisture patterns in a forested catchment: A hydropedological perspective. Geoderma 131, 345368. https://doi.org/10.1016/j.geoderma.2005.03.013</t>
         </is>
       </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>Cole_Farm</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2203,6 +2328,11 @@
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>Colpach</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2265,6 +2395,11 @@
         </is>
       </c>
       <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>Wollefsbach</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2323,6 +2458,11 @@
         </is>
       </c>
       <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>Angelo</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2385,6 +2525,11 @@
           <t>Lovill, S. M., Hahm, W. J., &amp; Dietrich, W. E. (2018). Drainage from the critical zone: Lithologic controls on the persistence and spatial extent of wetted channels during the summer dry season. Water Resources Research, 54(8), 5702â€“5726. https://doi.org/10.1029/2017wr021903</t>
         </is>
       </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>Sagehorn</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2449,6 +2594,11 @@
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>Maimai_catchments</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2507,6 +2657,11 @@
         </is>
       </c>
       <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>Mahurangi_catchments</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2565,6 +2720,11 @@
         </is>
       </c>
       <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Alptal</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2627,6 +2787,11 @@
         </is>
       </c>
       <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>Triple_G</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2685,6 +2850,11 @@
         </is>
       </c>
       <c r="P34" t="inlineStr"/>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>Zhurucay_Ecohydrological_Observatory</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2749,6 +2919,11 @@
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>A_in_Cofre_de_Perote_volcano</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2811,6 +2986,11 @@
           <t>Ocampo, Carlos J, Murugesu Sivapalan, and Carolyn E Oldham, 2006. â€œField Exploration of Coupled Hydrological and Biogeochemical Catchment Responses and a Unifying Perceptual Model.â€ Advances in Water Resources 29, no. 2 (2006): 161â€“80.</t>
         </is>
       </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>SB2_subcatchment</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2869,6 +3049,11 @@
         </is>
       </c>
       <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>Sumatra</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2935,6 +3120,11 @@
         </is>
       </c>
       <c r="P38" t="inlineStr"/>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>Hitachi_Ohta</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2993,6 +3183,11 @@
         </is>
       </c>
       <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>Baker_Creek</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3055,6 +3250,11 @@
         </is>
       </c>
       <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>Tatsunokuchi-yama_Forest</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3113,6 +3313,11 @@
         </is>
       </c>
       <c r="P41" t="inlineStr"/>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>Wolf_Creek</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3175,6 +3380,11 @@
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>Krycklan</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3237,6 +3447,11 @@
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>Girnock</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3299,6 +3514,11 @@
           <t>Uchida T, Asano Y, Ohte N, Mizuyama T. 2003. Analysis of flowpath dynamics in a steep unchannelled hollow in the Tanakami Mountains of Japan. Hydrological Processes 17 (2): 417â€“430 DOI: 10.1002/hyp.1133</t>
         </is>
       </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>Fudoji</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3357,6 +3577,11 @@
         </is>
       </c>
       <c r="P45" t="inlineStr"/>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>Dornbirnerach</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3415,6 +3640,11 @@
         </is>
       </c>
       <c r="P46" t="inlineStr"/>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>Gail</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3473,6 +3703,11 @@
         </is>
       </c>
       <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>Wimitzbach</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3531,6 +3766,11 @@
         </is>
       </c>
       <c r="P48" t="inlineStr"/>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>Perschling</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3601,6 +3841,11 @@
         </is>
       </c>
       <c r="P49" t="inlineStr"/>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>UhlÃÅskÃ</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3659,6 +3904,11 @@
         </is>
       </c>
       <c r="P50" t="inlineStr"/>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>Mulian</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3723,6 +3973,11 @@
           <t>Wenninger J, Uhlenbrook S, Lorentz S, Leibundgut C. 2008. Identification of runoff generation processes using combined hydrometric, tracer and geophysical methods in a headwater catchment in South Africa / Identification des processus de gÃ©nÃ©ration de lâ€™Ã©coulement par combinaison de mÃ©thodes hydromÃ©triques, de traÃ§age et gÃ©ophysiques dans un bassin versant sud-africain. Hydrological Sciences Journal 53 (2): 500â€“500 DOI: 10.1623/hysj.53.2.500</t>
         </is>
       </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>Weatherley</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3789,6 +4044,11 @@
           <t>Butzen, V., Seeger, M., Wirtz, S., Huemann, M., Mueller, C., Casper, M., Ries, J.B., 2014. Quantification of Hortonian overland flow generation and soil erosion in a Central European low mountain range using rainfall experiments. Catena 113, 202212. https://doi.org/10.1016/j.catena.2013.07.008</t>
         </is>
       </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>Huewelerbach_catchments</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3883,6 +4143,11 @@
 Antonelli, M., Glaser, B., Teuling, A.J., Klaus, J., Pfister, L., 2020a. Saturated areas through the lens: 1. Spatio-temporal variability of surface saturation documented through thermal infrared imagery. Hydrological Processes, 34: 13101332. https://doi.org/10.1002/hyp.13698</t>
         </is>
       </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>Weierbach</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3949,6 +4214,11 @@
           <t>Xiao, Xiong, Fan Zhang, Xiaoyan Li, Chen Zeng, Xiaonan Shi, Huawu Wu, Muhammad Dodo Jagirani, and Tao Che, 2020. â€œUsing Stable Isotopes to Identify Major Flow Pathways in a Permafrost Influenced Alpine Meadow Hillslope during Summer Rainfall Period.â€ Hydrological Processes 34, no. 5 (2020): 1104â€“16.</t>
         </is>
       </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>Yakou</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4007,6 +4277,11 @@
         </is>
       </c>
       <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>Longxi</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4069,6 +4344,11 @@
         </is>
       </c>
       <c r="P56" t="inlineStr"/>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>Duke_Forest_Research</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4131,6 +4411,11 @@
         </is>
       </c>
       <c r="P57" t="inlineStr"/>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>Rio_Vauz</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -4193,6 +4478,11 @@
         </is>
       </c>
       <c r="P58" t="inlineStr"/>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>Neversink</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -4255,6 +4545,11 @@
         </is>
       </c>
       <c r="P59" t="inlineStr"/>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>Moss_subwatershed</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -4313,6 +4608,11 @@
         </is>
       </c>
       <c r="P60" t="inlineStr"/>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>Walker_branch</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -4379,6 +4679,11 @@
           <t>Banks, Edward W, Craig T Simmons, Andrew J Love, Roger Cranswick, Adrian D Werner, Erick A Bestland, Martin Wood, and Tania Wilson, 2009. â€œFractured Bedrock and Saprolite Hydrogeologic Controls on Groundwater/Surface-Water Interaction: A Conceptual Model (Australia).â€ Hydrogeology Journal 17, no. 8 (2009): 1969â€“89.</t>
         </is>
       </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>Scott_Creek</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -4453,6 +4758,11 @@
           <t>Noguchi, S., Nik, A.R., Kasran, B., Tani, M., Sammori, T. and Morisada, K., 1997. Soil physical properties and preferential flow pathways in tropical rain forest, Bukit Tarek, Peninsular Malaysia. Journal of Forest Research, 2(2), pp.115-120.</t>
         </is>
       </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>Bukit_Tarek</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4521,6 +4831,11 @@
           <t>Katsuyama, M., Ohte, N., Kobashi, S., 2001. A three?component end?member analysis of streamwater hydrochemistry in a small Japanese forested headwater catchment. Hydrological Processes 15, 249260. https://doi.org/10.1002/hyp.155</t>
         </is>
       </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>Kiryu</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -4591,6 +4906,11 @@
         </is>
       </c>
       <c r="P64" t="inlineStr"/>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>Los_Alamos_National_Laboratorys_Environmental_Research_Park</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -4649,6 +4969,11 @@
         </is>
       </c>
       <c r="P65" t="inlineStr"/>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>Feshie</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -4719,6 +5044,11 @@
         </is>
       </c>
       <c r="P66" t="inlineStr"/>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>Sleepers</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -4777,6 +5107,11 @@
         </is>
       </c>
       <c r="P67" t="inlineStr"/>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>Saddle</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -4839,6 +5174,11 @@
           <t>Koch, J.C., Kikuchi, C.P., Wickland, K.P. and Schuster, P., 2014. Runoff sources and flow paths in a partially burned, upland boreal catchment underlain by permafrost. Water Resources Research, 50(10), pp.8141-8158.</t>
         </is>
       </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>West_Twin_Creek</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -4909,6 +5249,11 @@
           <t>Amatya, D.M.; Campbell, J.; Wohlgemuth, P.; Elder, K.; Sebestyen, S.; Johnson, S.; Keppeler, E.; Adams, M.B.; Caldwell, P.; and Misra, D. 2016. Hydrological processes of reference watersheds in Experimental Forests, USA. In: Forest Hydrology: Processes, Management, and Applications, Amatya, Williams, Bren, and de Jong (Editors), CABI Publishers, UK, pp: 219-239. 21 p.</t>
         </is>
       </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>Marcell</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -4971,6 +5316,11 @@
           <t>Hartmann, A., Kralik, M., Humer, F., Lange, J. and Weiler, M., 2012. Identification of a karst systemâ€™s intrinsic hydrodynamic parameters: upscaling from single springs to the whole aquifer. Environmental Earth Sciences, 65, pp.2377-2389.</t>
         </is>
       </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>Zoebelbodem</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -5029,6 +5379,11 @@
         </is>
       </c>
       <c r="P71" t="inlineStr"/>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>Hulu</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -5095,6 +5450,11 @@
           <t>Guida, D., Cuomo, A., Longobardi, A. and Villani, P., 2020. Geohydrology of a Reference Mediterranean Catchment (Cilento UNESCO Geopark, Southern Italy). Applied Sciences, 10(12), p.4117.</t>
         </is>
       </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>Ciciriello</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -5153,6 +5513,11 @@
         </is>
       </c>
       <c r="P73" t="inlineStr"/>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>Havikpak_Creek</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -5211,6 +5576,11 @@
         </is>
       </c>
       <c r="P74" t="inlineStr"/>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>Two_Boat_Lake</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -5269,6 +5639,11 @@
         </is>
       </c>
       <c r="P75" t="inlineStr"/>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>Upper_Jhelum</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -5327,6 +5702,11 @@
         </is>
       </c>
       <c r="P76" t="inlineStr"/>
+      <c r="Q76" t="inlineStr">
+        <is>
+          <t>Goodwater_Creek</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -5385,6 +5765,11 @@
         </is>
       </c>
       <c r="P77" t="inlineStr"/>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t>Mae_Sa_Noi</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -5447,6 +5832,11 @@
           <t>Vyse, S.A., Taie Semiromi, M., Lischeid, G. and Merz, C., 2020. Characterizing hydrological processes within kettle holes using stable water isotopes in the Uckermark of northern Brandenburg, Germany. Hydrological Processes, 34(8), pp.1868-1887.</t>
         </is>
       </c>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>Quillow</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -5509,6 +5899,11 @@
           <t>Zhao, P., Tang, X., Zhao, P., Zhang, W. and Tang, J., 2016. Mixing of event and preâ€event water in a shallow Entisol in sloping farmland based on isotopic and hydrometric measurements, SW China. Hydrological Processes, 30(19), pp.3478-3493.</t>
         </is>
       </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>Purple_soil</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -5567,6 +5962,11 @@
         </is>
       </c>
       <c r="P80" t="inlineStr"/>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>Heart_CZO</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -5625,6 +6025,11 @@
         </is>
       </c>
       <c r="P81" t="inlineStr"/>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>Mukeng</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -5687,6 +6092,11 @@
           <t>Ross, C. A., Ali, G., Bansah, S. &amp; Laing, J. R. (2017) Evaluating the Relative Importance of Shallow Subsurface Flow in a Prairie Landscape. Vadose Zone J. 16(5), 1â€“20. GeoScienceWorld. doi:10.2136/vzj2016.10.0096</t>
         </is>
       </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>Catfish_Creek</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -5745,6 +6155,11 @@
         </is>
       </c>
       <c r="P83" t="inlineStr"/>
+      <c r="Q83" t="inlineStr">
+        <is>
+          <t>San_Diego</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -5803,6 +6218,11 @@
         </is>
       </c>
       <c r="P84" t="inlineStr"/>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t>Thames_at_Kingston</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -5865,6 +6285,11 @@
           <t>Macpherson, G.L. and Sophocleous, M., 2004. Fast ground-water mixing and basal recharge in an unconfined, alluvial aquifer, Konza LTER Site, Northeastern Kansas. Journal of Hydrology, 286(1-4), pp.271-299.</t>
         </is>
       </c>
+      <c r="Q85" t="inlineStr">
+        <is>
+          <t>Konza_Prairie_LTER</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -5923,6 +6348,11 @@
         </is>
       </c>
       <c r="P86" t="inlineStr"/>
+      <c r="Q86" t="inlineStr">
+        <is>
+          <t>Peyto_Glacier_Research</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -5981,6 +6411,11 @@
         </is>
       </c>
       <c r="P87" t="inlineStr"/>
+      <c r="Q87" t="inlineStr">
+        <is>
+          <t>Samoylov_Island</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -6043,6 +6478,11 @@
           <t>Munk, L.A., Boutt, D.F., Moran, B.J., McKnight, S.V. and Jenckes, J., 2021. Hydrogeologic and Geochemical Distinctions in Freshwaterâ€Brine Systems of an Andean Salar. Geochemistry, Geophysics, Geosystems, 22(3), p.e2020GC009345.</t>
         </is>
       </c>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>Salar_de_Atacama</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -6101,6 +6541,11 @@
         </is>
       </c>
       <c r="P89" t="inlineStr"/>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>Tapado</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -6159,6 +6604,11 @@
         </is>
       </c>
       <c r="P90" t="inlineStr"/>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t>Santa_Elena_Ophiolite</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -6217,6 +6667,11 @@
         </is>
       </c>
       <c r="P91" t="inlineStr"/>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t>Dry_Lake</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -6279,6 +6734,11 @@
           <t>Koit, O., Tarros, S., PÃ¤rn, J., KÃ¼ttim, M., Abreldaal, P., Sisask, K., Vainu, M., Terasmaa, J., Retike, I. and Polikarpus, M., 2021. Contribution of local factors to the status of a groundwater dependent terrestrial ecosystem in the transboundary Gauja-Koiva River basin, North-Eastern Europe. Journal of Hydrology, 600, p.126656.</t>
         </is>
       </c>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t>Matsi_spring_fen</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -6337,6 +6797,11 @@
         </is>
       </c>
       <c r="P93" t="inlineStr"/>
+      <c r="Q93" t="inlineStr">
+        <is>
+          <t>TG_Halli</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -6395,6 +6860,11 @@
         </is>
       </c>
       <c r="P94" t="inlineStr"/>
+      <c r="Q94" t="inlineStr">
+        <is>
+          <t>Pallas</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -6453,6 +6923,11 @@
         </is>
       </c>
       <c r="P95" t="inlineStr"/>
+      <c r="Q95" t="inlineStr">
+        <is>
+          <t>Burabay_National_Nature_Park</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -6515,6 +6990,11 @@
           <t>Lesack LFW. 1993. Water balance and hydrologic characteristics of a rain forest catchment in the Central Amazon Basin. Water resources research 29 (3): 759â€“773 DOI: 10.1029/92wr02371</t>
         </is>
       </c>
+      <c r="Q96" t="inlineStr">
+        <is>
+          <t>Drainage_of_Lake_Calado</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -6573,6 +7053,11 @@
         </is>
       </c>
       <c r="P97" t="inlineStr"/>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>4_sub-basins_of_BanabuiuÌ</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -6631,6 +7116,11 @@
         </is>
       </c>
       <c r="P98" t="inlineStr"/>
+      <c r="Q98" t="inlineStr">
+        <is>
+          <t>Forquilha</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -6693,6 +7183,11 @@
           <t>Eger GZS, Silva Junior GC, Marques EAG, LeÃ£o BRC, da Rocha DGTB, Gilmore TE, do Amaral LGH, Silva JAO, Neale C. 2021. Recharge assessment in the context of expanding agricultural activity: Urucuia Aquifer System, western State of Bahia, Brazil. Journal of South American earth sciences 112 (103601): 103601 DOI: 10.1016/j.jsames.2021.103601</t>
         </is>
       </c>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t>Urucuia_Aquifer_system</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -6751,6 +7246,11 @@
         </is>
       </c>
       <c r="P100" t="inlineStr"/>
+      <c r="Q100" t="inlineStr">
+        <is>
+          <t>Upper_Ramuschaka</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -6813,6 +7313,11 @@
           <t>Ledford, S.H. and Lautz, L.K., 2015. Floodplain connection buffers seasonal changes in urban stream water quality. Hydrological processes, 29(6), pp.1002-1016.</t>
         </is>
       </c>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t>Meadowbrook_Creek</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -6871,6 +7376,11 @@
         </is>
       </c>
       <c r="P102" t="inlineStr"/>
+      <c r="Q102" t="inlineStr">
+        <is>
+          <t>Jatunhuaycu_Observatory</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -6933,6 +7443,11 @@
           <t>Mokua, R.A., Glenday, J., Nel, J. and Butler, M., 2020. Combined use of stable isotopes and hydrochemical characteristics to determine streamflow sources in the Jonkershoek catchment, South Africa. Isotopes in Environmental and Health Studies, 56(3), pp.238-259.</t>
         </is>
       </c>
+      <c r="Q103" t="inlineStr">
+        <is>
+          <t>Jonkershoek</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -6991,6 +7506,11 @@
         </is>
       </c>
       <c r="P104" t="inlineStr"/>
+      <c r="Q104" t="inlineStr">
+        <is>
+          <t>Zachariashoek_research_catchments</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -7049,6 +7569,11 @@
         </is>
       </c>
       <c r="P105" t="inlineStr"/>
+      <c r="Q105" t="inlineStr">
+        <is>
+          <t>CP-III</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -7111,6 +7636,11 @@
           <t>Harrison, R., van Tol, J. and Amiotte Suchet, P., 2022. Hydropedological Characteristics of the Cathedral Peak Research Catchments. Hydrology, 9(11), p.189.</t>
         </is>
       </c>
+      <c r="Q106" t="inlineStr">
+        <is>
+          <t>CP-IX</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -7169,6 +7699,11 @@
         </is>
       </c>
       <c r="P107" t="inlineStr"/>
+      <c r="Q107" t="inlineStr">
+        <is>
+          <t>CP-VI</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -7231,6 +7766,11 @@
         </is>
       </c>
       <c r="P108" t="inlineStr"/>
+      <c r="Q108" t="inlineStr">
+        <is>
+          <t>Fukuroyamasawa_B</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -7289,6 +7829,11 @@
         </is>
       </c>
       <c r="P109" t="inlineStr"/>
+      <c r="Q109" t="inlineStr">
+        <is>
+          <t>Nsimi</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -7347,6 +7892,11 @@
         </is>
       </c>
       <c r="P110" t="inlineStr"/>
+      <c r="Q110" t="inlineStr">
+        <is>
+          <t>Ene-Chilala</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -7405,6 +7955,11 @@
         </is>
       </c>
       <c r="P111" t="inlineStr"/>
+      <c r="Q111" t="inlineStr">
+        <is>
+          <t>Experim_Lakes_Area</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -7467,6 +8022,11 @@
           <t>Amatya, D.M.; Campbell, J.; Wohlgemuth, P.; Elder, K.; Sebestyen, S.; Johnson, S.; Keppeler, E.; Adams, M.B.; Caldwell, P.; and Misra, D. 2016. Hydrological processes of reference watersheds in Experimental Forests, USA. In: Forest Hydrology: Processes, Management, and Applications, Amatya, Williams, Bren, and de Jong (Editors), CABI Publishers, UK, pp: 219-239. 21 p.</t>
         </is>
       </c>
+      <c r="Q112" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -7529,6 +8089,11 @@
           <t>Amatya, D.M.; Campbell, J.; Wohlgemuth, P.; Elder, K.; Sebestyen, S.; Johnson, S.; Keppeler, E.; Adams, M.B.; Caldwell, P.; and Misra, D. 2016. Hydrological processes of reference watersheds in Experimental Forests, USA. In: Forest Hydrology: Processes, Management, and Applications, Amatya, Williams, Bren, and de Jong (Editors), CABI Publishers, UK, pp: 219-239. 21 p.</t>
         </is>
       </c>
+      <c r="Q113" t="inlineStr">
+        <is>
+          <t>Casper_Creek</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -7609,6 +8174,11 @@
           <t>Hudson, D.T., Leach, J.A., Webster, K., Houle, D., 2021. Streamflow regime of a lake?stream system based on long?term data from a high?density hydrometric network. Hydrological Processes 35, e14396. https://doi.org/10.1002/hyp.14396</t>
         </is>
       </c>
+      <c r="Q114" t="inlineStr">
+        <is>
+          <t>Coweeta</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -7681,6 +8251,11 @@
 Bates, N.S., Smith, J.A., Villarini, G., 2015. Flood response for the watersheds of the Fernow Experimental Forest in the central Appalachians. Water Resources Research 51, 44314453. https://doi.org/10.1002/2014WR015871</t>
         </is>
       </c>
+      <c r="Q115" t="inlineStr">
+        <is>
+          <t>Fernow</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -7743,6 +8318,11 @@
           <t>Amatya, D.M.; Campbell, J.; Wohlgemuth, P.; Elder, K.; Sebestyen, S.; Johnson, S.; Keppeler, E.; Adams, M.B.; Caldwell, P.; and Misra, D. 2016. Hydrological processes of reference watersheds in Experimental Forests, USA. In: Forest Hydrology: Processes, Management, and Applications, Amatya, Williams, Bren, and de Jong (Editors), CABI Publishers, UK, pp: 219-239. 21 p.</t>
         </is>
       </c>
+      <c r="Q116" t="inlineStr">
+        <is>
+          <t>Fraser</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -7825,6 +8405,11 @@
 Detty, J.M., McGuire, K.J., 2010. Topographic controls on shallow groundwater dynamics: implications of hydrologic connectivity between hillslopes and riparian zones in a till mantled catchment. Hydrological Processes 24, 22222236. https://doi.org/10.1002/hyp.7656</t>
         </is>
       </c>
+      <c r="Q117" t="inlineStr">
+        <is>
+          <t>Hubbard_Brook</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -7883,6 +8468,11 @@
         </is>
       </c>
       <c r="P118" t="inlineStr"/>
+      <c r="Q118" t="inlineStr">
+        <is>
+          <t>San_Dimas</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -7949,6 +8539,11 @@
           <t>Amatya, D.M.; Campbell, J.; Wohlgemuth, P.; Elder, K.; Sebestyen, S.; Johnson, S.; Keppeler, E.; Adams, M.B.; Caldwell, P.; and Misra, D. 2016. Hydrological processes of reference watersheds in Experimental Forests, USA. In: Forest Hydrology: Processes, Management, and Applications, Amatya, Williams, Bren, and de Jong (Editors), CABI Publishers, UK, pp: 219-239. 21 p.</t>
         </is>
       </c>
+      <c r="Q119" t="inlineStr">
+        <is>
+          <t>Santee</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -8007,6 +8602,11 @@
         </is>
       </c>
       <c r="P120" t="inlineStr"/>
+      <c r="Q120" t="inlineStr">
+        <is>
+          <t>Russell_Creek_Research</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -8065,6 +8665,11 @@
         </is>
       </c>
       <c r="P121" t="inlineStr"/>
+      <c r="Q121" t="inlineStr">
+        <is>
+          <t>Lemon</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -8129,6 +8734,11 @@
           <t>Ye, W., Bates, B.C., Viney, N.R., Sivapalan, M. and Jakeman, A.J., 1997. Performance of conceptual rainfallâ€runoff models in lowâ€yielding ephemeral catchments. Water Resources Research, 33(1), pp.153-166.</t>
         </is>
       </c>
+      <c r="Q122" t="inlineStr">
+        <is>
+          <t>Salmon_Brook</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -8191,6 +8801,11 @@
           <t>Becker, Alfred, and Jeffrey J McDonnell, 1998. â€œTopographical and Ecological Controls of Runoff Generation and Lateral Flows in Mountain Catchments.â€ Hydrology, Water Resources and Ecology in Headwaters, no. 248 (1998): 199.</t>
         </is>
       </c>
+      <c r="Q123" t="inlineStr">
+        <is>
+          <t>Schafertal</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -8255,6 +8870,11 @@
         </is>
       </c>
       <c r="P124" t="inlineStr"/>
+      <c r="Q124" t="inlineStr">
+        <is>
+          <t>MAT_subcatchment</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -8323,6 +8943,11 @@
           <t>Birch, Andrew L, Robert F Stallard, and Holly R Barnard, 2021. â€œPrecipitation Characteristics and Land Cover Control Wet Season Runoff Source and Rainfall Partitioning in Three Humid Tropical Catchments in Central Panama.â€ Water Resources Research 57, no. 2 (2021): e2020WR028058.</t>
         </is>
       </c>
+      <c r="Q125" t="inlineStr">
+        <is>
+          <t>SEC_subcatchment</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -8391,6 +9016,11 @@
           <t>Birch, Andrew L, Robert F Stallard, and Holly R Barnard, 2021. â€œPrecipitation Characteristics and Land Cover Control Wet Season Runoff Source and Rainfall Partitioning in Three Humid Tropical Catchments in Central Panama.â€ Water Resources Research 57, no. 2 (2021): e2020WR028058.</t>
         </is>
       </c>
+      <c r="Q126" t="inlineStr">
+        <is>
+          <t>PAS_subcatchment</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -8459,6 +9089,11 @@
           <t>Blume, Theresa, Erwin Zehe, Dominik E Reusser, AndrÃ©s IroumÃ©, and Axel Bronstert, 2008. â€œInvestigation of Runoff Generation in a Pristine, Poorly Gauged Catchment in the Chilean Andes I: A Multi-Method Experimental Study.â€ Hydrological Processes: An International Journal 22, no. 18 (2008): 3661â€“75.</t>
         </is>
       </c>
+      <c r="Q127" t="inlineStr">
+        <is>
+          <t>Malalcahuello</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -8537,6 +9172,11 @@
           <t>Bonell, M, and JM Fritsch, 1997. â€œCombining Hydrometric-Hydrochemistry Methods: A Challenge for Advancing Runoff Generation Process.â€ Hydrochemistry, no. 244 (1997): 165.</t>
         </is>
       </c>
+      <c r="Q128" t="inlineStr">
+        <is>
+          <t>South_Creek</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -8599,6 +9239,11 @@
           <t>Brown, V.A., McDonnell, J.J., Burns, D.A. and Kendall, C., 1999. The role of event water, a rapid shallow flow component, and catchment size in summer stormflow. Journal of Hydrology, 217(3-4), pp.171-190.</t>
         </is>
       </c>
+      <c r="Q129" t="inlineStr">
+        <is>
+          <t>Shelter_Creek</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -8657,6 +9302,11 @@
         </is>
       </c>
       <c r="P130" t="inlineStr"/>
+      <c r="Q130" t="inlineStr">
+        <is>
+          <t>Kaap</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -8725,6 +9375,11 @@
 Carey, SK, and WL Quinton, 2004. â€œEvaluating Snowmelt Runoff Generation in a Discontinuous Permafrost Catchment Using Stable Isotope, Hydrochemical and Hydrometric Data.â€ Hydrology Research 35, no. 4â€“5 (2004): 309â€“24.</t>
         </is>
       </c>
+      <c r="Q131" t="inlineStr">
+        <is>
+          <t>Granger</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -8783,6 +9438,11 @@
         </is>
       </c>
       <c r="P132" t="inlineStr"/>
+      <c r="Q132" t="inlineStr">
+        <is>
+          <t>Bukit_Timah</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -8845,6 +9505,11 @@
         </is>
       </c>
       <c r="P133" t="inlineStr"/>
+      <c r="Q133" t="inlineStr">
+        <is>
+          <t>W8S5</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -8911,6 +9576,11 @@
           <t>Chaves, J., Neill, C., Germer, S., Neto, S.G., Krusche, A. and Elsenbeer, H., 2008. Land management impacts on runoff sources in small Amazon watersheds. Hydrological Processes: An International Journal, 22(12), pp.1766-1775.</t>
         </is>
       </c>
+      <c r="Q134" t="inlineStr">
+        <is>
+          <t>Forest</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -8973,6 +9643,11 @@
           <t>Dahlke, Helen E, Steve W Lyon, Peter Jansson, TorbjÃ¶rn Karlin, and Gunhild Rosqvist, 2014\. â€œIsotopic Investigation of Runoff Generation in a Glacierized Catchment in Northern Sweden.â€ Hydrological Processes 28, no. 3 (2014): 1383â€“98.</t>
         </is>
       </c>
+      <c r="Q135" t="inlineStr">
+        <is>
+          <t>Tarfala</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -9035,6 +9710,11 @@
           <t>De Moraes, J.M., Schuler, A.E., Dunne, T., Figueiredo, R.D.O. and Victoria, R.L., 2006. Water storage and runoff processes in plinthic soils under forest and pasture in eastern Amazonia. Hydrological Processes: An International Journal, 20(12), pp.2509-2526.</t>
         </is>
       </c>
+      <c r="Q136" t="inlineStr">
+        <is>
+          <t>Forest_catchment_Fazenda_Vitoria</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -9105,6 +9785,11 @@
           <t>Elsenbeer, H. and Lack, A., 1996. Hydrometric and hydrochemicai evidence for fast flowpaths at La Cuenca, Western Amazonia. Journal of Hydrology, 180(1-4), pp.237-250.</t>
         </is>
       </c>
+      <c r="Q137" t="inlineStr">
+        <is>
+          <t>La_Cuenca</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -9171,6 +9856,11 @@
           <t>Flerchinger, G.N., Cooley, K.R. and Ralston, D.R., 1992. Groundwater response to snowmelt in a mountainous watershed. Journal of Hydrology, 133(3-4), pp.293-311.</t>
         </is>
       </c>
+      <c r="Q138" t="inlineStr">
+        <is>
+          <t>Upper_Sheep_Creek</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -9233,6 +9923,11 @@
           <t>Freyberg, Jana von, P Suresh C Rao, Dirk Radny, and Mario Schirmer, 2015. â€œThe Impact of Hillslope Groundwater Dynamics and Landscape Functioning in Event-Flow Generation: A Field Study in the Rietholzbach Catchment, Switzerland.â€ Hydrogeology Journal 23, no. 5 (2015): 935â€“48.</t>
         </is>
       </c>
+      <c r="Q139" t="inlineStr">
+        <is>
+          <t>Rietholzbach</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -9311,6 +10006,11 @@
 Post, D.A., Jones, J.A., 2001. Hydrologic regimes of forested, mountainous, headwater basins in New Hampshire, North Carolina, Oregon, and Puerto Rico. Advances in Water Resources 24, 11951210. https://doi.org/10.1016/S0309-1708(01)00036-7</t>
         </is>
       </c>
+      <c r="Q140" t="inlineStr">
+        <is>
+          <t>WS3</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -9383,6 +10083,11 @@
 Soulsby, C., Scheliga, B., Neill, A., Comte, J.-C., &amp; Tetzlaff, D. (2021). A longer-term perspective on soil moisture, groundwater and stream flow response to the 2018 drought in an experimental catchment in the Scottish Highlands. Hydrological Processes, 35(6), e14206.</t>
         </is>
       </c>
+      <c r="Q141" t="inlineStr">
+        <is>
+          <t>Bruntland_Burn</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -9445,6 +10150,11 @@
           <t>Gibson, JJ, TWD Edwards, and TD Prowse, 1993. â€œRunoff Generation in a High Boreal Wetland in Northern Canada: Paper Presented at the 9th Northern Res. Basin Symposium/Workshop (Whitehorse/Dawson/Inuvik, Canada-August 1992).â€ Hydrology Research 24, no. 2â€“3 (1993): 213â€“24.</t>
         </is>
       </c>
+      <c r="Q142" t="inlineStr">
+        <is>
+          <t>Manners_Creek_tributary_site</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -9521,6 +10231,11 @@
 Zimmermann, A., Francke, T. and Elsenbeer, H., 2012. Forests and erosion: Insights from a study of suspended-sediment dynamics in an overland flow-prone rainforest catchment. Journal of Hydrology, 428, pp.170-181.</t>
         </is>
       </c>
+      <c r="Q143" t="inlineStr">
+        <is>
+          <t>Lutz_Creek</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -9583,6 +10298,11 @@
         </is>
       </c>
       <c r="P144" t="inlineStr"/>
+      <c r="Q144" t="inlineStr">
+        <is>
+          <t>Conrad_Trail_Stream</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -9649,6 +10369,11 @@
         </is>
       </c>
       <c r="P145" t="inlineStr"/>
+      <c r="Q145" t="inlineStr">
+        <is>
+          <t>Rancho_Grande</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -9711,6 +10436,11 @@
         </is>
       </c>
       <c r="P146" t="inlineStr"/>
+      <c r="Q146" t="inlineStr">
+        <is>
+          <t>Rio_San_Francisco</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -9773,6 +10503,11 @@
         </is>
       </c>
       <c r="P147" t="inlineStr"/>
+      <c r="Q147" t="inlineStr">
+        <is>
+          <t>Hemuqiao</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -9835,6 +10570,11 @@
           <t>Haugen, R.K., Slaughter, C.W., Howe, K.E. and Dingman, S.L., 1982. Hydrology and climatology of the Caribou-Poker creeks research watershed, Alaska. COLD REGIONS RESEARCH AND ENGINEERING LAB HANOVER NH.</t>
         </is>
       </c>
+      <c r="Q148" t="inlineStr">
+        <is>
+          <t>C1-3</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -9893,6 +10633,11 @@
         </is>
       </c>
       <c r="P149" t="inlineStr"/>
+      <c r="Q149" t="inlineStr">
+        <is>
+          <t>Caribou-Poker</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -9951,6 +10696,11 @@
         </is>
       </c>
       <c r="P150" t="inlineStr"/>
+      <c r="Q150" t="inlineStr">
+        <is>
+          <t>Zastler</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -10027,6 +10777,11 @@
           <t>Fuss, C.B., Driscoll, C.T., Green, M.B., Groffman, P.M., 2016. Hydrologic flowpaths during snowmelt in forested headwater catchments under differing winter climatic and soil frost regimes. Hydrological Processes 30, 46174632. https://doi.org/10.1002/hyp.10956</t>
         </is>
       </c>
+      <c r="Q151" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -10089,6 +10844,11 @@
           <t>Hughes, Justin D, Shahbaz Khan, Russell S Crosbie, Stuart Helliwell, and David L Michalk, 2007. â€œRunoff and Solute Mobilization Processes in a Semiarid Headwater Catchment.â€ Water Resources Research 43, no. 9 (2007).</t>
         </is>
       </c>
+      <c r="Q152" t="inlineStr">
+        <is>
+          <t>Brays_Flat_Creek</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -10155,6 +10915,11 @@
         </is>
       </c>
       <c r="P153" t="inlineStr"/>
+      <c r="Q153" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -10217,6 +10982,11 @@
           <t>Jin, Zhao, Li Guo, Yunlong Yu, Da Luo, Bihang Fan, and Guangchen Chu, 2020. â€œStorm Runoff Generation in Headwater Catchments on the Chinese Loess Plateau after Long-Term Vegetation Rehabilitation.â€ Science of the Total Environment 748 (2020): 141375.</t>
         </is>
       </c>
+      <c r="Q154" t="inlineStr">
+        <is>
+          <t>Nanxiaohe</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -10275,6 +11045,11 @@
         </is>
       </c>
       <c r="P155" t="inlineStr"/>
+      <c r="Q155" t="inlineStr">
+        <is>
+          <t>Oxisol_and_Ultisol_watersheds</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -10337,6 +11112,11 @@
           <t>Johnson, Mark S, William F Coon, Vishal K Mehta, Tammo S Steenhuis, Erin S Brooks, and Jan Boll, 2003. â€œApplication of Two Hydrologic Models with Different Runoff Mechanisms to a Hillslope Dominated Watershed in the Northeastern US: A Comparison of HSPF and SMR.â€ Journal of Hydrology 284, no. 1â€“4 (2003): 57â€“76.</t>
         </is>
       </c>
+      <c r="Q156" t="inlineStr">
+        <is>
+          <t>Irondequoit_Creek</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -10399,6 +11179,11 @@
           <t>Kim, Jin Kwan, Yuichi Onda, Min Seok Kim, and Dong Yoon Yang, 2014. â€œPlot-Scale Study of Surface Runoff on Well-Covered Forest Floors under Different Canopy Species.â€ Quaternary International 344 (2014): 75â€“85.</t>
         </is>
       </c>
+      <c r="Q157" t="inlineStr">
+        <is>
+          <t>Woldong</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -10457,6 +11242,11 @@
         </is>
       </c>
       <c r="P158" t="inlineStr"/>
+      <c r="Q158" t="inlineStr">
+        <is>
+          <t>Hakyuchi</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -10521,6 +11311,11 @@
         </is>
       </c>
       <c r="P159" t="inlineStr"/>
+      <c r="Q159" t="inlineStr">
+        <is>
+          <t>Turkey_Creek_WS_78</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -10583,6 +11378,11 @@
         </is>
       </c>
       <c r="P160" t="inlineStr"/>
+      <c r="Q160" t="inlineStr">
+        <is>
+          <t>Strengbach</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -10645,6 +11445,11 @@
           <t>Laine-Kaulio, Hanne, Soile BacknÃ¤s, Harri Koivusalo, and Ari LaurÃ©n, 2015. â€œDye Tracer Visualization of Flow Patterns and Pathways in Glacial Sandy till at a Boreal Forest Hillslope.â€ Geoderma 259 (2015): 23â€“34.</t>
         </is>
       </c>
+      <c r="Q161" t="inlineStr">
+        <is>
+          <t>Kangaslampi</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -10703,6 +11508,11 @@
         </is>
       </c>
       <c r="P162" t="inlineStr"/>
+      <c r="Q162" t="inlineStr">
+        <is>
+          <t>Deir_Ibzei</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -10779,6 +11589,11 @@
 Latron, J., Gallart, F., 1995. Hydrological response of two nested small Mediterranean basins presenting various degradation states. Physics and Chemistry of the Earth 20, 369374. https://doi.org/10.1016/0079-1946(95)00050-X</t>
         </is>
       </c>
+      <c r="Q163" t="inlineStr">
+        <is>
+          <t>Can_Vila</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -10841,6 +11656,11 @@
           <t>Lindenmaier, FALK, ERWIN Zehe, MARTIN Helms, O Evadakov, and JÃ¼rgen Ihringer, 2006. â€œEffect of Soil Shrinkage on Runoff Generation in Micro and Mesoscale Catchments.â€ IAHS PUBLICATION 303 (2006): 305.</t>
         </is>
       </c>
+      <c r="Q164" t="inlineStr">
+        <is>
+          <t>Tannhausen</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -10899,6 +11719,11 @@
         </is>
       </c>
       <c r="P165" t="inlineStr"/>
+      <c r="Q165" t="inlineStr">
+        <is>
+          <t>Bull_and_Providence_catchments</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -10961,6 +11786,11 @@
           <t>Liu, F., Parmenter, R., Brooks, P.D., Conklin, M.H. and Bales, R.C., 2008. Seasonal and interannual variation of streamflow pathways and biogeochemical implications in semiâ€arid, forested catchments in Valles Caldera, New Mexico. Ecohydrology: Ecosystems, Land and Water Process Interactions, Ecohydrogeomorphology, 1(3), pp.239-252.</t>
         </is>
       </c>
+      <c r="Q166" t="inlineStr">
+        <is>
+          <t>Valles_Caldera</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -11019,6 +11849,11 @@
         </is>
       </c>
       <c r="P167" t="inlineStr"/>
+      <c r="Q167" t="inlineStr">
+        <is>
+          <t>Martinelli</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -11077,6 +11912,11 @@
         </is>
       </c>
       <c r="P168" t="inlineStr"/>
+      <c r="Q168" t="inlineStr">
+        <is>
+          <t>GL4</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -11135,6 +11975,11 @@
         </is>
       </c>
       <c r="P169" t="inlineStr"/>
+      <c r="Q169" t="inlineStr">
+        <is>
+          <t>Sustenpass</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -11203,6 +12048,11 @@
 SÃ¡nchezâ€Murillo, R., Romeroâ€Esquivel, L.G., JimÃ©nezâ€AntillÃn, J., Salasâ€Navarro, J., Corralesâ€Salazar, L., Ãlvarezâ€Carvajal, J., Ãlvarezâ€McInerney, S., Bonillaâ€Barrantes, D., GutiÃ©rrezâ€Sibaja, N., MartÃ­nezâ€Arroyo, M. and Ortizâ€Apuy, E., 2019. DOC transport and export in a dynamic tropical catchment. Journal of Geophysical Research: Biogeosciences, 124(6), pp.1665-1679.</t>
         </is>
       </c>
+      <c r="Q170" t="inlineStr">
+        <is>
+          <t>Cerro_Dantas</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -11265,6 +12115,11 @@
           <t>McCaig, Michael, 1983. â€œContributions to Storm Quickflow in a Small Headwater Catchmentâ€”the Role of Natural Pipes and Soil Macropores.â€ Earth Surface Processes and Landforms 8, no. 3 (1983): 239â€“52.</t>
         </is>
       </c>
+      <c r="Q171" t="inlineStr">
+        <is>
+          <t>Slithero_Clough</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -11327,6 +12182,11 @@
           <t>McDaniel, P. A., Regan, M. P., Brooks, E., Boll, J., Barndt, S., Falen, A., et al. (2008). Linking fragipans, perched water tables, and catchment-scale hydrological processes. Catena, 73(2), 166â€“173.</t>
         </is>
       </c>
+      <c r="Q172" t="inlineStr">
+        <is>
+          <t>Troy</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -11385,6 +12245,11 @@
         </is>
       </c>
       <c r="P173" t="inlineStr"/>
+      <c r="Q173" t="inlineStr">
+        <is>
+          <t>Upper_Dry_Creek</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -11463,6 +12328,11 @@
 Miyata, S., Kosugi, K., Nishi, Y., Gomi, T., Sidle, R.C., Mizuyama, T., 2010. Spatial pattern of infiltration rate and its effect on hydrological processes in a small headwater catchment. Hydrological Processes 24, 535549. https://doi.org/10.1002/hyp.7549</t>
         </is>
       </c>
+      <c r="Q174" t="inlineStr">
+        <is>
+          <t>Hinotani-ike</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -11521,6 +12391,11 @@
         </is>
       </c>
       <c r="P175" t="inlineStr"/>
+      <c r="Q175" t="inlineStr">
+        <is>
+          <t>Migina</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -11583,6 +12458,11 @@
           <t>Nunes, JoÃ£o Pedro, LÃ©onard Bernard-Jannin, Maria Luz Rodriguez Blanco, Juliana Marisa Santos, Celeste de Oliveira Alves Coelho, and Jan Jacob Keizer, 2018. â€œHydrological and Erosion Processes in Terraced Fields: Observations from a Humid Mediterranean Region in Northern Portugal.â€ Land Degradation &amp; Development 29, no. 3 (2018): 596â€“606.</t>
         </is>
       </c>
+      <c r="Q176" t="inlineStr">
+        <is>
+          <t>Macieira_de_AlcÃba</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -11645,6 +12525,11 @@
           <t>Onda, Yuichi, Maki Tsujimura, Jun-ichi Fujihara, and Jun Ito, 2006. â€œRunoff Generation Mechanisms in High-Relief Mountainous Watersheds with Different Underlying Geology.â€ Journal of Hydrology 331, no. 3â€“4 (2006): 659â€“73.</t>
         </is>
       </c>
+      <c r="Q177" t="inlineStr">
+        <is>
+          <t>Ina</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -11703,6 +12588,11 @@
         </is>
       </c>
       <c r="P178" t="inlineStr"/>
+      <c r="Q178" t="inlineStr">
+        <is>
+          <t>VÃne</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -11761,6 +12651,11 @@
         </is>
       </c>
       <c r="P179" t="inlineStr"/>
+      <c r="Q179" t="inlineStr">
+        <is>
+          <t>PC1-08_Plastic_Lake</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -11835,6 +12730,11 @@
           <t>Hudson, D.T., Leach, J.A., Webster, K., Houle, D., 2021. Streamflow regime of a lake?stream system based on long?term data from a high?density hydrometric network. Hydrological Processes 35, e14396. https://doi.org/10.1002/hyp.14396</t>
         </is>
       </c>
+      <c r="Q180" t="inlineStr">
+        <is>
+          <t>W2</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -11915,6 +12815,11 @@
 Detty, J.M., McGuire, K.J., 2010. Topographic controls on shallow groundwater dynamics: implications of hydrologic connectivity between hillslopes and riparian zones in a till mantled catchment. Hydrological Processes 24, 22222236. https://doi.org/10.1002/hyp.7656</t>
         </is>
       </c>
+      <c r="Q181" t="inlineStr">
+        <is>
+          <t>WS1</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -11977,6 +12882,11 @@
           <t>Post, D.A. and Jones, J.A., 2001. Hydrologic regimes of forested, mountainous, headwater basins in New Hampshire, North Carolina, Oregon, and Puerto Rico. Advances in Water Resources, 24(9-10), pp.1195-1210.</t>
         </is>
       </c>
+      <c r="Q182" t="inlineStr">
+        <is>
+          <t>Bisley</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -12049,6 +12959,11 @@
 Quinton, WL, M Hayashi, and LE Chasmer, 2009. â€œPeatland Hydrology of Discontinuous Permafrost in the Northwest Territories: Overview and Synthesis.â€ Canadian Water Resources Journal 34, no. 4 (2009): 311â€“28.</t>
         </is>
       </c>
+      <c r="Q183" t="inlineStr">
+        <is>
+          <t>Scotty_Creek</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -12111,6 +13026,11 @@
           <t>Scheffler, R., Neill, C., Krusche, A.V. and Elsenbeer, H., 2011. Soil hydraulic response to land-use change associated with the recent soybean expansion at the Amazon agricultural frontier. Agriculture, Ecosystems &amp; Environment, 144(1), pp.281-289.</t>
         </is>
       </c>
+      <c r="Q184" t="inlineStr">
+        <is>
+          <t>Tanguro</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -12169,6 +13089,11 @@
         </is>
       </c>
       <c r="P185" t="inlineStr"/>
+      <c r="Q185" t="inlineStr">
+        <is>
+          <t>Bisley_II</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -12227,6 +13152,11 @@
         </is>
       </c>
       <c r="P186" t="inlineStr"/>
+      <c r="Q186" t="inlineStr">
+        <is>
+          <t>Sand_Mountain_Research_and_Station</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -12311,6 +13241,11 @@
 Hudson, D.T., Leach, J.A., Webster, K., Houle, D., 2021. Streamflow regime of a lake?stream system based on long?term data from a high?density hydrometric network. Hydrological Processes 35, e14396. https://doi.org/10.1002/hyp.14396</t>
         </is>
       </c>
+      <c r="Q187" t="inlineStr">
+        <is>
+          <t>WS02</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -12373,6 +13308,11 @@
           <t>Sklash, M.G. and Farvolden, R.N., 1979. The role of groundwater in storm runoff. Journal of Hydrology, 43(1-4), pp.45-65.</t>
         </is>
       </c>
+      <c r="Q188" t="inlineStr">
+        <is>
+          <t>Ruisseau_des_Eaux_Volees</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -12435,6 +13375,11 @@
           <t>Soulsby, Chris, and Sarah M Dunn, 2003. â€œTowards Integrating Tracer Studies in Conceptual Rainfall-Runoff Models: Recent Insights from a Sub-Arctic Catchment in the Cairngorm Mountains, Scotland.â€ Hydrological Processes 17, no. 2 (2003): 403â€“16.</t>
         </is>
       </c>
+      <c r="Q189" t="inlineStr">
+        <is>
+          <t>Allt_aâ_Mharcaidh</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -12493,6 +13438,11 @@
         </is>
       </c>
       <c r="P190" t="inlineStr"/>
+      <c r="Q190" t="inlineStr">
+        <is>
+          <t>Ll1_control</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -12565,6 +13515,11 @@
 Uchida, T., Tromp-van Meerveld, I., McDonnell, J.J., 2005. The role of lateral pipe flow in hillslope runoff response: an intercomparison of non-linear hillslope response. Journal of Hydrology 311, 117133. https://doi.org/10.1016/j.jhydrol.2005.01.012</t>
         </is>
       </c>
+      <c r="Q191" t="inlineStr">
+        <is>
+          <t>Toinotani</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -12627,6 +13582,11 @@
           <t>Wan, Chengwei, Kai Li, Huili Zhang, Zhongbo Yu, Peng Yi, and Chenghao Chen, 2020. â€œIntegrating Isotope Mass Balance and Water Residence Time Dating: Insights of Runoff Generation in Small Permafrost Watersheds from Stable and Radioactive Isotopes.â€ Journal of Radioanalytical and Nuclear Chemistry 326, no. 1 (2020): 241â€“54.</t>
         </is>
       </c>
+      <c r="Q192" t="inlineStr">
+        <is>
+          <t>SAYR</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -12685,6 +13645,11 @@
         </is>
       </c>
       <c r="P193" t="inlineStr"/>
+      <c r="Q193" t="inlineStr">
+        <is>
+          <t>Nucice</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -12743,6 +13708,11 @@
         </is>
       </c>
       <c r="P194" t="inlineStr"/>
+      <c r="Q194" t="inlineStr">
+        <is>
+          <t>Chezine</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -12801,6 +13771,11 @@
         </is>
       </c>
       <c r="P195" t="inlineStr"/>
+      <c r="Q195" t="inlineStr">
+        <is>
+          <t>WeiÃŸeritz</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -12859,6 +13834,11 @@
         </is>
       </c>
       <c r="P196" t="inlineStr"/>
+      <c r="Q196" t="inlineStr">
+        <is>
+          <t>Hupsel_Brook</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -12921,6 +13901,11 @@
           <t>Bonell, M., Pearce, A.J. and Stewart, M.K., 1990. The identification of runoffâ€production mechanisms using environmental isotopes in a tussock grassland catchment, eastern Otago, New Zealand. Hydrological Processes, 4(1), pp.15-34.</t>
         </is>
       </c>
+      <c r="Q197" t="inlineStr">
+        <is>
+          <t>Glendhu_catchments</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -12983,6 +13968,11 @@
           <t>Taylor, C.H. and Pearce, A.J., 1982. Storm runoff processes and subcatchment characteristics in a New Zealand hill country catchment. Earth Surface Processes and Landforms, 7(5), pp.439-447.</t>
         </is>
       </c>
+      <c r="Q198" t="inlineStr">
+        <is>
+          <t>Hut_Creek</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -13053,6 +14043,11 @@
           <t>Penna, D., van Meerveld, H.J., Oliviero, O., Zuecco, G., Assendelft, R.S., Dalla Fontana, G. and Borga, M.A.R.C.O., 2015. Seasonal changes in runoff generation in a small forested mountain catchment. Hydrological Processes, 29(8), pp.2027-2042.</t>
         </is>
       </c>
+      <c r="Q199" t="inlineStr">
+        <is>
+          <t>Ressi</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -13111,6 +14106,11 @@
         </is>
       </c>
       <c r="P200" t="inlineStr"/>
+      <c r="Q200" t="inlineStr">
+        <is>
+          <t>Hilly_Ecosystem_Research_Station</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -13169,6 +14169,11 @@
         </is>
       </c>
       <c r="P201" t="inlineStr"/>
+      <c r="Q201" t="inlineStr">
+        <is>
+          <t>Haute-Mentue</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -13231,6 +14236,11 @@
           <t>MartÃ­nezâ€Mena, M., Albaladejo, J. and Castillo, V.M., 1998. Factors influencing surface runoff generation in a Mediterranean semiâ€arid environment: Chicamo watershed, SE Spain. Hydrological processes, 12(5), pp.741-754.</t>
         </is>
       </c>
+      <c r="Q202" t="inlineStr">
+        <is>
+          <t>Chicamo</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -13289,6 +14299,11 @@
         </is>
       </c>
       <c r="P203" t="inlineStr"/>
+      <c r="Q203" t="inlineStr">
+        <is>
+          <t>Pukemanga_Stream</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -13347,6 +14362,11 @@
         </is>
       </c>
       <c r="P204" t="inlineStr"/>
+      <c r="Q204" t="inlineStr">
+        <is>
+          <t>Harra</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -13405,6 +14425,11 @@
         </is>
       </c>
       <c r="P205" t="inlineStr"/>
+      <c r="Q205" t="inlineStr">
+        <is>
+          <t>Grasslands_Research_Station</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -13467,6 +14492,11 @@
         </is>
       </c>
       <c r="P206" t="inlineStr"/>
+      <c r="Q206" t="inlineStr">
+        <is>
+          <t>Baratz</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -13525,6 +14555,11 @@
         </is>
       </c>
       <c r="P207" t="inlineStr"/>
+      <c r="Q207" t="inlineStr">
+        <is>
+          <t>Yayama</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -13587,6 +14622,11 @@
           <t>George, R.J. and Conacher, A.J. (1993), Mechanisms responsible for streamflow generation on a small, salt-affected and deeply weathered hillslope. Earth Surf. Process. Landforms, 18: 291-309.</t>
         </is>
       </c>
+      <c r="Q208" t="inlineStr">
+        <is>
+          <t>Narrogin</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -13649,6 +14689,11 @@
           <t>KuraÅ›, P.K., Weiler, M. and Alila, Y., 2008. The spatiotemporal variability of runoff generation and groundwater dynamics in a snow-dominated catchment. Journal of Hydrology, 352(1-2), pp.50-66.</t>
         </is>
       </c>
+      <c r="Q209" t="inlineStr">
+        <is>
+          <t>Upper_Penticton_Creek_Experiment</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -13707,6 +14752,11 @@
         </is>
       </c>
       <c r="P210" t="inlineStr"/>
+      <c r="Q210" t="inlineStr">
+        <is>
+          <t>N04D</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -13765,6 +14815,11 @@
         </is>
       </c>
       <c r="P211" t="inlineStr"/>
+      <c r="Q211" t="inlineStr">
+        <is>
+          <t>ArnÃs</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -13823,6 +14878,11 @@
         </is>
       </c>
       <c r="P212" t="inlineStr"/>
+      <c r="Q212" t="inlineStr">
+        <is>
+          <t>Mâb_Ìe</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -13885,6 +14945,11 @@
           <t>PesÃ¡ntez, J., Birkel, C., Mosquera, G.M., CÃ©lleri, R., Contreras, P., CÃ¡rdenas, I. and Crespo, P., 2023. Bridging the gap from hydrological to biogeochemical processes using tracer-aided hydrological models in a tropical montane ecosystem. Journal of Hydrology, p.129328.</t>
         </is>
       </c>
+      <c r="Q213" t="inlineStr">
+        <is>
+          <t>Subcatchment_of_Zhurucay_Ecohydrological_Observatory</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -13943,6 +15008,11 @@
         </is>
       </c>
       <c r="P214" t="inlineStr"/>
+      <c r="Q214" t="inlineStr">
+        <is>
+          <t>Coet_Dan</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -14001,6 +15071,11 @@
         </is>
       </c>
       <c r="P215" t="inlineStr"/>
+      <c r="Q215" t="inlineStr">
+        <is>
+          <t>Aglar</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -14059,6 +15134,11 @@
         </is>
       </c>
       <c r="P216" t="inlineStr"/>
+      <c r="Q216" t="inlineStr">
+        <is>
+          <t>Archer_Creek</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -14119,6 +15199,11 @@
         </is>
       </c>
       <c r="P217" t="inlineStr"/>
+      <c r="Q217" t="inlineStr">
+        <is>
+          <t>Aiuaba</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -14177,6 +15262,11 @@
         </is>
       </c>
       <c r="P218" t="inlineStr"/>
+      <c r="Q218" t="inlineStr">
+        <is>
+          <t>RBF_subcatchment</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -14239,6 +15329,11 @@
           <t>Ross SM, Thornes JB, Nortcliff S. 1990. Soil hydrology, nutrient and erosional response to the clearance of Terra Firme forest, maraca island, Roraima, northern Brazil. The geographical journal 156 (3): 267 DOI: 10.2307/635528</t>
         </is>
       </c>
+      <c r="Q219" t="inlineStr">
+        <is>
+          <t>The_terra_firme_forest_of_Maraca_Island</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -14303,6 +15398,11 @@
           <t>de Barros CAP, Govers G, Minella JPG, Ramon R. 2021. How water flow components affect sediment dynamics modeling in a Brazilian catchment. Journal of hydrology 597 (126111): 126111 DOI: 10.1016/j.jhydrol.2021.126111</t>
         </is>
       </c>
+      <c r="Q220" t="inlineStr">
+        <is>
+          <t>Lajeado_Ferreira</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -14361,6 +15461,11 @@
         </is>
       </c>
       <c r="P221" t="inlineStr"/>
+      <c r="Q221" t="inlineStr">
+        <is>
+          <t>Cumaru</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -14419,6 +15524,11 @@
         </is>
       </c>
       <c r="P222" t="inlineStr"/>
+      <c r="Q222" t="inlineStr">
+        <is>
+          <t>Jianpinggou</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -14477,6 +15587,11 @@
         </is>
       </c>
       <c r="P223" t="inlineStr"/>
+      <c r="Q223" t="inlineStr">
+        <is>
+          <t>San_Lorencito_headwater</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -14535,6 +15650,11 @@
         </is>
       </c>
       <c r="P224" t="inlineStr"/>
+      <c r="Q224" t="inlineStr">
+        <is>
+          <t>El_Morro</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -14597,6 +15717,11 @@
           <t>Perez, A.B., Innocente dos Santos, C., SÃ¡, J.H., Arienti, P.F. and Chaffe, P.L., 2020. Connectivity of ephemeral and intermittent streams in a subtropical Atlantic forest headwater catchment. Water, 12(6), p.1526.</t>
         </is>
       </c>
+      <c r="Q225" t="inlineStr">
+        <is>
+          <t>Retiro_headwater</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -14655,6 +15780,11 @@
         </is>
       </c>
       <c r="P226" t="inlineStr"/>
+      <c r="Q226" t="inlineStr">
+        <is>
+          <t>Walnut_Gulch</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -14713,6 +15843,11 @@
         </is>
       </c>
       <c r="P227" t="inlineStr"/>
+      <c r="Q227" t="inlineStr">
+        <is>
+          <t>Little</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -14771,6 +15906,11 @@
         </is>
       </c>
       <c r="P228" t="inlineStr"/>
+      <c r="Q228" t="inlineStr">
+        <is>
+          <t>Obere_Brachtpe</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -14829,6 +15969,11 @@
         </is>
       </c>
       <c r="P229" t="inlineStr"/>
+      <c r="Q229" t="inlineStr">
+        <is>
+          <t>Bohlmicke</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -14891,6 +16036,11 @@
           <t>MeiÃŸl, G, Formayer, H, Klebinder, K, et al, 2017. Climate change effects on hydrological system conditions influencing generation of storm runoff in small Alpine catchments. Hydrological Processes. 2017; 31: 1314â€“1330.</t>
         </is>
       </c>
+      <c r="Q230" t="inlineStr">
+        <is>
+          <t>Ruggbach</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -14949,6 +16099,11 @@
         </is>
       </c>
       <c r="P231" t="inlineStr"/>
+      <c r="Q231" t="inlineStr">
+        <is>
+          <t>Brixenbach</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -15007,6 +16162,11 @@
         </is>
       </c>
       <c r="P232" t="inlineStr"/>
+      <c r="Q232" t="inlineStr">
+        <is>
+          <t>LÃngentalbach</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -15069,6 +16229,11 @@
           <t>Burt, TP, Worrall, F, Howden, NJK, Jarvie, HP, Pratt, A, Hutchinson, TH, 2021. A 50-year record of nitrate concentrations in the Slapton Ley Catchment, Devon, United Kingdom. Hydrological Processes. 2021; 35:e13955.</t>
         </is>
       </c>
+      <c r="Q233" t="inlineStr">
+        <is>
+          <t>Slapton_Wood</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -15137,6 +16302,11 @@
 Hudson, D.T., Leach, J.A., Webster, K., Houle, D., 2021. Streamflow regime of a lake?stream system based on long?term data from a high?density hydrometric network. Hydrological Processes 35, e14396. https://doi.org/10.1002/hyp.14396</t>
         </is>
       </c>
+      <c r="Q234" t="inlineStr">
+        <is>
+          <t>Turkey_Lakes</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -15199,6 +16369,11 @@
           <t>Coltharp, G. &amp; Springer, Everett. (1980). Hydrologic Characteristics of an Undisturbed Hardwood Watershed in Eastern Kentucky. Conference: Central hardwoods Conference III September 16-17, 1980</t>
         </is>
       </c>
+      <c r="Q235" t="inlineStr">
+        <is>
+          <t>Falling_Rock</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -15265,6 +16440,11 @@
           <t>Holko, L, Danko, M, Sleziak, P, 2021. Snowmelt characteristics in a pristine mountain catchment of the JaloveckÃ½ Creek, Slovakia, over the last three decades. Hydrological Processes. 2021; 35:e14128.</t>
         </is>
       </c>
+      <c r="Q236" t="inlineStr">
+        <is>
+          <t>JaloveckÃ½_Creek</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -15327,6 +16507,11 @@
           <t>Ledesma, J. L. J., Lupon, A., &amp; Bernal, S. (2021). Hydrological responses to rainfall events including the extratropical cyclone Gloria in two contrasting Mediterranean headwaters in Spain; the perennial font del RegÃ s and the intermittent Fuirosos. Hydrological Processes, 35(12), e14451</t>
         </is>
       </c>
+      <c r="Q237" t="inlineStr">
+        <is>
+          <t>Font_del_RegÃ_s</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -15389,6 +16574,11 @@
           <t>Ledesma, J. L. J., Lupon, A., &amp; Bernal, S. (2021). Hydrological responses to rainfall events including the extratropical cyclone Gloria in two contrasting Mediterranean headwaters in Spain; the perennial font del RegÃ s and the intermittent Fuirosos. Hydrological Processes, 35(12), e14452</t>
         </is>
       </c>
+      <c r="Q238" t="inlineStr">
+        <is>
+          <t>Fuirosos</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -15447,6 +16637,11 @@
         </is>
       </c>
       <c r="P239" t="inlineStr"/>
+      <c r="Q239" t="inlineStr">
+        <is>
+          <t>Oak_Ridge_Reservation</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -15505,6 +16700,11 @@
         </is>
       </c>
       <c r="P240" t="inlineStr"/>
+      <c r="Q240" t="inlineStr">
+        <is>
+          <t>Upper_Kuparuk</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -15563,6 +16763,11 @@
         </is>
       </c>
       <c r="P241" t="inlineStr"/>
+      <c r="Q241" t="inlineStr">
+        <is>
+          <t>Mule_Hole</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -15621,6 +16826,11 @@
         </is>
       </c>
       <c r="P242" t="inlineStr"/>
+      <c r="Q242" t="inlineStr">
+        <is>
+          <t>Ratier</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -15683,6 +16893,11 @@
           <t>Jones, J.A.A. (1987), The effects of soil piping on contributing areas and erosion patterns. Earth Surf. Process. Landforms, 12: 229-248</t>
         </is>
       </c>
+      <c r="Q243" t="inlineStr">
+        <is>
+          <t>Maesnant</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -15743,6 +16958,11 @@
       <c r="P244" t="inlineStr">
         <is>
           <t>Myrabø, S., 1986. Runoff Studies in a Small Catchment: Paper presented at the Nordic Hydrological Conference (Reykjavik, Iceland, August–1986). Hydrology Research, 17(4-5), pp.335-346.</t>
+        </is>
+      </c>
+      <c r="Q244" t="inlineStr">
+        <is>
+          <t>Asker</t>
         </is>
       </c>
     </row>

</xml_diff>